<commit_message>
nas folders script working
</commit_message>
<xml_diff>
--- a/Templates/Shamiya Expansion - Inventory Tracking v1.11.xlsx
+++ b/Templates/Shamiya Expansion - Inventory Tracking v1.11.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/825aabd020ed0793/Projects/foreman/Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/50d76e1b4061cd6b/Thales/GIT/foreman/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="207" documentId="8_{E36932E3-75BD-4B4D-87E8-57AD0925E03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{438BF435-A627-4965-B807-227F7AC0C32A}"/>
+  <xr:revisionPtr revIDLastSave="217" documentId="8_{E36932E3-75BD-4B4D-87E8-57AD0925E03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96ECB881-5630-4896-910C-F88FDB6E607C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="610" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="610" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -166,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6613" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6617" uniqueCount="786">
   <si>
     <t>Hardware Type</t>
   </si>
@@ -2529,6 +2529,12 @@
   </si>
   <si>
     <t>Rack Placement</t>
+  </si>
+  <si>
+    <t>SV-MTR-0305-11E-08</t>
+  </si>
+  <si>
+    <t>11E</t>
   </si>
 </sst>
 </file>
@@ -3525,18 +3531,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="16.54296875" customWidth="1"/>
-    <col min="2" max="2" width="34.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5546875" customWidth="1"/>
+    <col min="2" max="2" width="34.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="86.453125" customWidth="1"/>
+    <col min="5" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="86.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1"/>
-    <row r="2" spans="1:7" ht="14.5" customHeight="1" thickBot="1">
+    <row r="2" spans="1:7" ht="14.55" customHeight="1" thickBot="1">
       <c r="A2" s="23" t="s">
         <v>0</v>
       </c>
@@ -3628,7 +3634,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="43.5">
+    <row r="6" spans="1:7" ht="43.2">
       <c r="A6" s="43" t="s">
         <v>1</v>
       </c>
@@ -3651,7 +3657,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="58">
+    <row r="7" spans="1:7" ht="57.6">
       <c r="A7" s="43" t="s">
         <v>2</v>
       </c>
@@ -3674,7 +3680,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="43.5">
+    <row r="8" spans="1:7" ht="43.2">
       <c r="A8" s="43" t="s">
         <v>3</v>
       </c>
@@ -3749,14 +3755,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="B1:G20"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="15" thickBot="1"/>
@@ -4013,27 +4019,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:V481"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="42.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.7265625" customWidth="1"/>
+    <col min="1" max="1" width="42.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" customWidth="1"/>
-    <col min="6" max="6" width="4.26953125" customWidth="1"/>
-    <col min="7" max="7" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" customWidth="1"/>
+    <col min="6" max="6" width="4.21875" customWidth="1"/>
+    <col min="7" max="7" width="7.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="10" width="29" customWidth="1"/>
-    <col min="11" max="11" width="17.81640625" customWidth="1"/>
-    <col min="12" max="12" width="15.81640625" customWidth="1"/>
-    <col min="13" max="13" width="61.7265625" customWidth="1"/>
-    <col min="14" max="15" width="18.26953125" customWidth="1"/>
-    <col min="16" max="17" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.453125" customWidth="1"/>
-    <col min="19" max="19" width="31.453125" customWidth="1"/>
-    <col min="20" max="20" width="13.453125" customWidth="1"/>
-    <col min="21" max="21" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.77734375" customWidth="1"/>
+    <col min="12" max="12" width="15.77734375" customWidth="1"/>
+    <col min="13" max="13" width="61.77734375" customWidth="1"/>
+    <col min="14" max="15" width="18.21875" customWidth="1"/>
+    <col min="16" max="17" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.44140625" customWidth="1"/>
+    <col min="19" max="19" width="31.44140625" customWidth="1"/>
+    <col min="20" max="20" width="13.44140625" customWidth="1"/>
+    <col min="21" max="21" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15" thickBot="1">
@@ -4404,7 +4410,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:22" hidden="1">
       <c r="A7" s="2" t="s">
         <v>760</v>
       </c>
@@ -4467,7 +4473,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:22" hidden="1">
       <c r="A8" s="2" t="s">
         <v>760</v>
       </c>
@@ -4656,7 +4662,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:22" hidden="1">
       <c r="A11" s="2" t="s">
         <v>760</v>
       </c>
@@ -5160,7 +5166,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:22" hidden="1">
       <c r="A19" s="2" t="s">
         <v>760</v>
       </c>
@@ -5286,7 +5292,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:22">
+    <row r="21" spans="1:22" hidden="1">
       <c r="A21" s="2" t="s">
         <v>760</v>
       </c>
@@ -8503,7 +8509,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="72" spans="1:22">
+    <row r="72" spans="1:22" hidden="1">
       <c r="A72" s="2" t="s">
         <v>760</v>
       </c>
@@ -11898,7 +11904,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="126" spans="1:22">
+    <row r="126" spans="1:22" hidden="1">
       <c r="A126" s="2" t="s">
         <v>760</v>
       </c>
@@ -11961,7 +11967,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="127" spans="1:22">
+    <row r="127" spans="1:22" hidden="1">
       <c r="A127" s="2" t="s">
         <v>760</v>
       </c>
@@ -12024,7 +12030,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="128" spans="1:22">
+    <row r="128" spans="1:22" hidden="1">
       <c r="A128" s="2" t="s">
         <v>760</v>
       </c>
@@ -12654,7 +12660,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="138" spans="1:22">
+    <row r="138" spans="1:22" hidden="1">
       <c r="A138" s="2" t="s">
         <v>760</v>
       </c>
@@ -14850,7 +14856,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="173" spans="1:22">
+    <row r="173" spans="1:22" hidden="1">
       <c r="A173" s="2" t="s">
         <v>760</v>
       </c>
@@ -14913,7 +14919,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="174" spans="1:22">
+    <row r="174" spans="1:22" hidden="1">
       <c r="A174" s="2" t="s">
         <v>760</v>
       </c>
@@ -15165,7 +15171,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="178" spans="1:22">
+    <row r="178" spans="1:22" hidden="1">
       <c r="A178" s="2" t="s">
         <v>760</v>
       </c>
@@ -15417,7 +15423,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="182" spans="1:22">
+    <row r="182" spans="1:22" hidden="1">
       <c r="A182" s="2" t="s">
         <v>760</v>
       </c>
@@ -18365,7 +18371,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="229" spans="1:22">
+    <row r="229" spans="1:22" hidden="1">
       <c r="A229" s="2" t="s">
         <v>760</v>
       </c>
@@ -18428,7 +18434,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="230" spans="1:22">
+    <row r="230" spans="1:22" hidden="1">
       <c r="A230" s="2" t="s">
         <v>760</v>
       </c>
@@ -18491,7 +18497,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="231" spans="1:22">
+    <row r="231" spans="1:22" hidden="1">
       <c r="A231" s="2" t="s">
         <v>760</v>
       </c>
@@ -18554,7 +18560,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="232" spans="1:22">
+    <row r="232" spans="1:22" hidden="1">
       <c r="A232" s="2" t="s">
         <v>760</v>
       </c>
@@ -18617,7 +18623,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="233" spans="1:22">
+    <row r="233" spans="1:22" hidden="1">
       <c r="A233" s="2" t="s">
         <v>760</v>
       </c>
@@ -18680,7 +18686,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="234" spans="1:22">
+    <row r="234" spans="1:22" hidden="1">
       <c r="A234" s="2" t="s">
         <v>760</v>
       </c>
@@ -18795,7 +18801,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="236" spans="1:22">
+    <row r="236" spans="1:22" hidden="1">
       <c r="A236" s="2" t="s">
         <v>760</v>
       </c>
@@ -18858,7 +18864,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="237" spans="1:22">
+    <row r="237" spans="1:22" hidden="1">
       <c r="A237" s="2" t="s">
         <v>760</v>
       </c>
@@ -18973,7 +18979,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="239" spans="1:22">
+    <row r="239" spans="1:22" hidden="1">
       <c r="A239" s="2" t="s">
         <v>760</v>
       </c>
@@ -19036,7 +19042,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="240" spans="1:22">
+    <row r="240" spans="1:22" hidden="1">
       <c r="A240" s="2" t="s">
         <v>760</v>
       </c>
@@ -19151,7 +19157,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="242" spans="1:22">
+    <row r="242" spans="1:22" hidden="1">
       <c r="A242" s="2" t="s">
         <v>760</v>
       </c>
@@ -19279,7 +19285,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="244" spans="1:22">
+    <row r="244" spans="1:22" hidden="1">
       <c r="A244" s="2" t="s">
         <v>760</v>
       </c>
@@ -19342,7 +19348,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="245" spans="1:22">
+    <row r="245" spans="1:22" hidden="1">
       <c r="A245" s="2" t="s">
         <v>760</v>
       </c>
@@ -22919,21 +22925,32 @@
         <v>37</v>
       </c>
     </row>
-    <row r="304" spans="1:22" hidden="1">
-      <c r="A304" s="2"/>
+    <row r="304" spans="1:22">
+      <c r="A304" s="2" t="s">
+        <v>760</v>
+      </c>
       <c r="B304" s="1"/>
-      <c r="C304" s="1"/>
-      <c r="D304" s="1"/>
-      <c r="E304" s="1"/>
+      <c r="C304" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D304" s="1">
+        <v>5</v>
+      </c>
+      <c r="E304" s="1">
+        <v>2</v>
+      </c>
       <c r="F304" s="1"/>
-      <c r="G304" s="1"/>
-      <c r="H304" s="1"/>
+      <c r="G304" s="1">
+        <v>8</v>
+      </c>
+      <c r="H304" s="1" t="s">
+        <v>784</v>
+      </c>
       <c r="I304" s="1" t="s">
-        <v>776</v>
-      </c>
-      <c r="J304" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v>ICE</v>
+        <v>532</v>
+      </c>
+      <c r="J304" s="1" t="s">
+        <v>785</v>
       </c>
       <c r="K304" s="1"/>
       <c r="L304" s="31" t="s">
@@ -25989,7 +26006,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="353" spans="1:22" hidden="1">
+    <row r="353" spans="1:22">
       <c r="A353" s="2" t="s">
         <v>760</v>
       </c>
@@ -27214,7 +27231,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="373" spans="1:22" hidden="1">
+    <row r="373" spans="1:22">
       <c r="A373" s="2" t="s">
         <v>760</v>
       </c>
@@ -27340,7 +27357,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="375" spans="1:22" hidden="1">
+    <row r="375" spans="1:22">
       <c r="A375" s="2" t="s">
         <v>760</v>
       </c>
@@ -27466,7 +27483,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="377" spans="1:22" hidden="1">
+    <row r="377" spans="1:22">
       <c r="A377" s="2" t="s">
         <v>760</v>
       </c>
@@ -27529,7 +27546,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="378" spans="1:22" hidden="1">
+    <row r="378" spans="1:22">
       <c r="A378" s="2" t="s">
         <v>760</v>
       </c>
@@ -27592,7 +27609,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="379" spans="1:22" hidden="1">
+    <row r="379" spans="1:22">
       <c r="A379" s="2" t="s">
         <v>760</v>
       </c>
@@ -27655,7 +27672,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="380" spans="1:22" hidden="1">
+    <row r="380" spans="1:22">
       <c r="A380" s="2" t="s">
         <v>760</v>
       </c>
@@ -32908,9 +32925,16 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:V474" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="3">
+    <filterColumn colId="7">
       <filters>
-        <filter val="13"/>
+        <filter val="SV-MTR-0305-11E-01"/>
+        <filter val="SV-MTR-0305-11E-02"/>
+        <filter val="SV-MTR-0305-11E-03"/>
+        <filter val="SV-MTR-0305-11E-04"/>
+        <filter val="SV-MTR-0305-11E-05"/>
+        <filter val="SV-MTR-0305-11E-06"/>
+        <filter val="SV-MTR-0305-11E-07"/>
+        <filter val="SV-MTR-0305-11E-08"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -32969,7 +32993,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D2B7418-72A8-445C-BF64-FC62E23BFFA5}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -33001,19 +33025,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:Q30"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="4" width="16.26953125" customWidth="1"/>
-    <col min="5" max="5" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1796875" customWidth="1"/>
-    <col min="7" max="7" width="13.453125" customWidth="1"/>
-    <col min="8" max="8" width="12.453125" hidden="1" customWidth="1"/>
-    <col min="9" max="10" width="19.26953125" customWidth="1"/>
+    <col min="3" max="4" width="16.21875" customWidth="1"/>
+    <col min="5" max="5" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.21875" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" hidden="1" customWidth="1"/>
+    <col min="9" max="10" width="19.21875" customWidth="1"/>
     <col min="11" max="11" width="58" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.7265625" customWidth="1"/>
+    <col min="15" max="15" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="29.5" thickBot="1">
+    <row r="1" spans="1:16" ht="29.4" thickBot="1">
       <c r="A1" s="51" t="s">
         <v>519</v>
       </c>
@@ -33046,7 +33070,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="29.5" hidden="1" thickBot="1">
+    <row r="2" spans="1:16" ht="29.4" hidden="1" thickBot="1">
       <c r="A2" s="64" t="s">
         <v>713</v>
       </c>
@@ -33690,7 +33714,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="29.5" hidden="1" thickBot="1">
+    <row r="22" spans="1:17" ht="29.4" hidden="1" thickBot="1">
       <c r="A22" s="2">
         <v>18</v>
       </c>
@@ -33735,7 +33759,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="29.5" hidden="1" thickBot="1">
+    <row r="23" spans="1:17" ht="29.4" hidden="1" thickBot="1">
       <c r="A23" s="2">
         <v>18</v>
       </c>
@@ -33776,7 +33800,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="29.5" hidden="1" thickBot="1">
+    <row r="24" spans="1:17" ht="29.4" hidden="1" thickBot="1">
       <c r="A24" s="2">
         <v>18</v>
       </c>
@@ -34039,18 +34063,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M31"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="3" width="16.26953125" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1796875" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.21875" customWidth="1"/>
+    <col min="6" max="6" width="13.44140625" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" customWidth="1"/>
     <col min="8" max="8" width="58" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.7265625" customWidth="1"/>
+    <col min="12" max="12" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="29.5" thickBot="1">
+    <row r="1" spans="1:13" ht="29.4" thickBot="1">
       <c r="A1" s="51" t="s">
         <v>519</v>
       </c>
@@ -34076,7 +34100,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="29.5" thickBot="1">
+    <row r="2" spans="1:13" ht="29.4" thickBot="1">
       <c r="A2" s="64" t="s">
         <v>713</v>
       </c>
@@ -34095,7 +34119,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="29">
+    <row r="3" spans="1:13" ht="28.8">
       <c r="A3" s="20">
         <v>18</v>
       </c>
@@ -34126,7 +34150,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="29">
+    <row r="4" spans="1:13" ht="28.8">
       <c r="A4" s="2">
         <v>18</v>
       </c>
@@ -34157,7 +34181,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="29">
+    <row r="5" spans="1:13" ht="28.8">
       <c r="A5" s="2">
         <v>18</v>
       </c>
@@ -34826,15 +34850,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="6.26953125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="6.21875" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="91" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="29">
+    <row r="1" spans="1:4" ht="28.8">
       <c r="A1" t="s">
         <v>730</v>
       </c>
@@ -34931,7 +34955,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="29">
+    <row r="12" spans="1:4" ht="28.8">
       <c r="B12" s="54" t="s">
         <v>739</v>
       </c>
@@ -35012,25 +35036,25 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:N33"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="26">
+    <row r="1" spans="1:14" ht="27.6">
       <c r="A1" s="26" t="s">
         <v>567</v>
       </c>
@@ -35074,7 +35098,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="26">
+    <row r="2" spans="1:14" ht="27.6">
       <c r="A2" s="26" t="s">
         <v>579</v>
       </c>
@@ -35118,7 +35142,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="26">
+    <row r="3" spans="1:14" ht="27.6">
       <c r="A3" s="26" t="s">
         <v>591</v>
       </c>
@@ -35162,7 +35186,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="26">
+    <row r="4" spans="1:14" ht="27.6">
       <c r="A4" s="26" t="s">
         <v>593</v>
       </c>
@@ -35206,7 +35230,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="26">
+    <row r="5" spans="1:14" ht="27.6">
       <c r="A5" s="26" t="s">
         <v>595</v>
       </c>
@@ -35250,7 +35274,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="26">
+    <row r="6" spans="1:14" ht="27.6">
       <c r="A6" s="26" t="s">
         <v>597</v>
       </c>
@@ -35294,7 +35318,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="26">
+    <row r="7" spans="1:14" ht="27.6">
       <c r="A7" s="26" t="s">
         <v>599</v>
       </c>
@@ -35338,7 +35362,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="26">
+    <row r="8" spans="1:14" ht="27.6">
       <c r="A8" s="26" t="s">
         <v>603</v>
       </c>
@@ -35382,7 +35406,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="26">
+    <row r="9" spans="1:14" ht="27.6">
       <c r="A9" s="26" t="s">
         <v>605</v>
       </c>
@@ -35426,7 +35450,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="26">
+    <row r="10" spans="1:14" ht="27.6">
       <c r="A10" s="26" t="s">
         <v>607</v>
       </c>
@@ -35470,7 +35494,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="26">
+    <row r="11" spans="1:14" ht="27.6">
       <c r="A11" s="26" t="s">
         <v>609</v>
       </c>
@@ -35514,7 +35538,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="26">
+    <row r="12" spans="1:14" ht="27.6">
       <c r="A12" s="26" t="s">
         <v>611</v>
       </c>
@@ -35558,7 +35582,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="26">
+    <row r="13" spans="1:14" ht="27.6">
       <c r="A13" s="26" t="s">
         <v>613</v>
       </c>
@@ -35602,7 +35626,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="26">
+    <row r="14" spans="1:14" ht="27.6">
       <c r="A14" s="26" t="s">
         <v>615</v>
       </c>
@@ -35646,7 +35670,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="26">
+    <row r="15" spans="1:14" ht="27.6">
       <c r="A15" s="26" t="s">
         <v>617</v>
       </c>
@@ -35690,7 +35714,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="26">
+    <row r="16" spans="1:14" ht="27.6">
       <c r="A16" s="26" t="s">
         <v>619</v>
       </c>
@@ -35734,7 +35758,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="26">
+    <row r="17" spans="1:14" ht="27.6">
       <c r="A17" s="26" t="s">
         <v>621</v>
       </c>
@@ -35778,7 +35802,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="26">
+    <row r="18" spans="1:14" ht="27.6">
       <c r="A18" s="26" t="s">
         <v>623</v>
       </c>
@@ -35822,7 +35846,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="26">
+    <row r="19" spans="1:14" ht="27.6">
       <c r="A19" s="26" t="s">
         <v>624</v>
       </c>
@@ -35866,7 +35890,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="26">
+    <row r="20" spans="1:14" ht="27.6">
       <c r="A20" s="26" t="s">
         <v>625</v>
       </c>
@@ -35910,7 +35934,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="26">
+    <row r="21" spans="1:14" ht="27.6">
       <c r="A21" s="26" t="s">
         <v>626</v>
       </c>
@@ -35954,7 +35978,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="26">
+    <row r="22" spans="1:14" ht="27.6">
       <c r="A22" s="26" t="s">
         <v>628</v>
       </c>
@@ -35998,7 +36022,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="26">
+    <row r="23" spans="1:14" ht="27.6">
       <c r="A23" s="26" t="s">
         <v>630</v>
       </c>
@@ -36042,7 +36066,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="26">
+    <row r="24" spans="1:14" ht="27.6">
       <c r="A24" s="26" t="s">
         <v>632</v>
       </c>
@@ -36086,7 +36110,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="26">
+    <row r="25" spans="1:14" ht="27.6">
       <c r="A25" s="26" t="s">
         <v>634</v>
       </c>
@@ -36130,7 +36154,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="26">
+    <row r="26" spans="1:14" ht="27.6">
       <c r="A26" s="26" t="s">
         <v>636</v>
       </c>
@@ -36174,7 +36198,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="26">
+    <row r="27" spans="1:14" ht="27.6">
       <c r="A27" s="26" t="s">
         <v>638</v>
       </c>
@@ -36218,7 +36242,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="26">
+    <row r="28" spans="1:14" ht="27.6">
       <c r="A28" s="26" t="s">
         <v>640</v>
       </c>
@@ -36262,7 +36286,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="26">
+    <row r="29" spans="1:14" ht="27.6">
       <c r="A29" s="26" t="s">
         <v>642</v>
       </c>
@@ -36306,7 +36330,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="26">
+    <row r="30" spans="1:14" ht="27.6">
       <c r="A30" s="26" t="s">
         <v>644</v>
       </c>
@@ -36350,7 +36374,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="26">
+    <row r="31" spans="1:14" ht="27.6">
       <c r="A31" s="26" t="s">
         <v>646</v>
       </c>
@@ -36394,7 +36418,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="26">
+    <row r="32" spans="1:14" ht="27.6">
       <c r="A32" s="26" t="s">
         <v>647</v>
       </c>
@@ -36438,7 +36462,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="26">
+    <row r="33" spans="1:14" ht="27.6">
       <c r="A33" s="26" t="s">
         <v>652</v>
       </c>
@@ -36495,13 +36519,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C107"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.7265625" customWidth="1"/>
+    <col min="1" max="1" width="17.77734375" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="33.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" thickBot="1">
@@ -37573,15 +37597,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB3372C1-1EB7-4865-B329-46380D9FCBE9}">
   <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="41" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="38.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="38.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="58">
+    <row r="1" spans="1:13" ht="57.6">
       <c r="A1" s="43" t="s">
         <v>1</v>
       </c>
@@ -37613,7 +37637,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="116">
+    <row r="2" spans="1:13" ht="115.2">
       <c r="A2" s="43" t="s">
         <v>2</v>
       </c>
@@ -37645,7 +37669,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="58">
+    <row r="3" spans="1:13" ht="57.6">
       <c r="A3" s="43" t="s">
         <v>3</v>
       </c>

</xml_diff>